<commit_message>
Revert back here maybe
</commit_message>
<xml_diff>
--- a/Predictions/2026-04-25.xlsx
+++ b/Predictions/2026-04-25.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gdsak\OneDrive\Desktop\Glicko-2, Etc\Predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5671FAC4-92D6-4649-B539-FA6BA943C3AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{668CC47F-1F04-42B3-A530-06448738C1E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Predictions" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="50">
   <si>
     <t>Red Corner</t>
   </si>
@@ -170,12 +170,6 @@
   </si>
   <si>
     <t>Old Model</t>
-  </si>
-  <si>
-    <t>Mean Duration (min)</t>
-  </si>
-  <si>
-    <t>Monte Carlo</t>
   </si>
 </sst>
 </file>
@@ -233,7 +227,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -251,6 +245,18 @@
         <fgColor rgb="FFD3D3D3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -377,7 +383,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -412,13 +418,6 @@
     <xf numFmtId="165" fontId="4" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -428,14 +427,61 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -452,34 +498,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -782,7 +807,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
@@ -801,36 +826,32 @@
     <col min="14" max="14" width="6.7109375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="19.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="D1" s="21" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="D1" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="21" t="s">
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="35" t="s">
         <v>49</v>
       </c>
-      <c r="L1" s="23"/>
-      <c r="M1" s="21" t="s">
+      <c r="L1" s="37"/>
+      <c r="M1" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="N1" s="23"/>
-      <c r="O1" s="24" t="s">
+      <c r="N1" s="37"/>
+      <c r="O1" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="P1" s="25"/>
-      <c r="Q1" s="20" t="s">
-        <v>51</v>
-      </c>
+      <c r="P1" s="39"/>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -876,14 +897,11 @@
       <c r="O2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="P2" s="17" t="s">
+      <c r="P2" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="Q2" s="18" t="s">
-        <v>50</v>
-      </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -914,29 +932,26 @@
       <c r="J3" s="9">
         <v>0.36499999999999999</v>
       </c>
-      <c r="K3" s="16" t="s">
+      <c r="K3" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="L3" s="15">
+      <c r="L3" s="12">
         <v>0.59860000000000002</v>
       </c>
-      <c r="M3" s="12" t="s">
+      <c r="M3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="N3" s="13">
+      <c r="N3" s="32">
         <v>0.66364661234241717</v>
       </c>
-      <c r="O3" s="12" t="s">
+      <c r="O3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="P3" s="14" t="s">
+      <c r="P3" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="Q3" s="19">
-        <v>12.45</v>
-      </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
@@ -946,50 +961,47 @@
       <c r="C4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="27">
+      <c r="E4" s="16">
         <v>0.63100000000000001</v>
       </c>
-      <c r="F4" s="28" t="s">
+      <c r="F4" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="27">
+      <c r="G4" s="16">
         <v>0.67200000000000004</v>
       </c>
-      <c r="H4" s="27">
+      <c r="H4" s="16">
         <v>0.67200000000000004</v>
       </c>
-      <c r="I4" s="27">
+      <c r="I4" s="16">
         <v>0.22</v>
       </c>
-      <c r="J4" s="29">
+      <c r="J4" s="18">
         <v>0.108</v>
       </c>
-      <c r="K4" s="30" t="s">
+      <c r="K4" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="L4" s="31">
+      <c r="L4" s="20">
         <v>0.53259999999999996</v>
       </c>
-      <c r="M4" s="32" t="s">
+      <c r="M4" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="N4" s="33">
+      <c r="N4" s="22">
         <v>0.64000470105801432</v>
       </c>
-      <c r="O4" s="32" t="s">
+      <c r="O4" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="P4" s="34" t="s">
+      <c r="P4" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="Q4" s="19">
-        <v>12.5</v>
-      </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -999,50 +1011,47 @@
       <c r="C5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="27">
+      <c r="E5" s="26">
         <v>0.69899999999999995</v>
       </c>
-      <c r="F5" s="28" t="s">
+      <c r="F5" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="27">
+      <c r="G5" s="26">
         <v>0.48</v>
       </c>
-      <c r="H5" s="27">
+      <c r="H5" s="26">
         <v>0.48</v>
       </c>
-      <c r="I5" s="27">
+      <c r="I5" s="26">
         <v>0.19800000000000001</v>
       </c>
-      <c r="J5" s="29">
+      <c r="J5" s="28">
         <v>0.32300000000000001</v>
       </c>
-      <c r="K5" s="30" t="s">
+      <c r="K5" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="L5" s="31">
+      <c r="L5" s="41">
         <v>0.51270000000000004</v>
       </c>
-      <c r="M5" s="32" t="s">
+      <c r="M5" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="N5" s="33">
+      <c r="N5" s="22">
         <v>0.5311204164831429</v>
       </c>
-      <c r="O5" s="26" t="s">
+      <c r="O5" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="P5" s="34" t="s">
+      <c r="P5" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="Q5" s="19">
-        <v>11.48</v>
-      </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>21</v>
       </c>
@@ -1052,50 +1061,47 @@
       <c r="C6" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="27">
+      <c r="E6" s="16">
         <v>0.63300000000000001</v>
       </c>
-      <c r="F6" s="28" t="s">
+      <c r="F6" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="27">
+      <c r="G6" s="16">
         <v>0.48299999999999998</v>
       </c>
-      <c r="H6" s="27">
+      <c r="H6" s="16">
         <v>0.48299999999999998</v>
       </c>
-      <c r="I6" s="27">
+      <c r="I6" s="16">
         <v>0.26800000000000002</v>
       </c>
-      <c r="J6" s="29">
+      <c r="J6" s="18">
         <v>0.249</v>
       </c>
-      <c r="K6" s="30" t="s">
+      <c r="K6" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="L6" s="31">
+      <c r="L6" s="41">
         <v>0.52490000000000003</v>
       </c>
-      <c r="M6" s="32" t="s">
+      <c r="M6" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="N6" s="33">
+      <c r="N6" s="30">
         <v>0.55716029124117272</v>
       </c>
-      <c r="O6" s="32" t="s">
+      <c r="O6" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="P6" s="34" t="s">
+      <c r="P6" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="Q6" s="19">
-        <v>10.6</v>
-      </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>24</v>
       </c>
@@ -1105,50 +1111,47 @@
       <c r="C7" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="27">
+      <c r="E7" s="16">
         <v>0.68</v>
       </c>
-      <c r="F7" s="28" t="s">
+      <c r="F7" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="27">
+      <c r="G7" s="16">
         <v>0.51900000000000002</v>
       </c>
-      <c r="H7" s="27">
+      <c r="H7" s="16">
         <v>0.51900000000000002</v>
       </c>
-      <c r="I7" s="27">
+      <c r="I7" s="16">
         <v>0.309</v>
       </c>
-      <c r="J7" s="29">
+      <c r="J7" s="18">
         <v>0.17199999999999999</v>
       </c>
-      <c r="K7" s="30" t="s">
+      <c r="K7" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="L7" s="31">
+      <c r="L7" s="20">
         <v>0.60209999999999997</v>
       </c>
-      <c r="M7" s="32" t="s">
+      <c r="M7" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="N7" s="33">
+      <c r="N7" s="22">
         <v>0.56002441810554782</v>
       </c>
-      <c r="O7" s="26" t="s">
+      <c r="O7" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="P7" s="34" t="s">
+      <c r="P7" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="Q7" s="19">
-        <v>11.42</v>
-      </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>26</v>
       </c>
@@ -1158,50 +1161,47 @@
       <c r="C8" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="27">
+      <c r="E8" s="16">
         <v>0.64900000000000002</v>
       </c>
-      <c r="F8" s="28" t="s">
+      <c r="F8" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="27">
+      <c r="G8" s="16">
         <v>0.47399999999999998</v>
       </c>
-      <c r="H8" s="27">
+      <c r="H8" s="16">
         <v>0.47399999999999998</v>
       </c>
-      <c r="I8" s="27">
+      <c r="I8" s="16">
         <v>0.40500000000000003</v>
       </c>
-      <c r="J8" s="29">
+      <c r="J8" s="18">
         <v>0.122</v>
       </c>
-      <c r="K8" s="30" t="s">
+      <c r="K8" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="L8" s="31">
+      <c r="L8" s="20">
         <v>0.5232</v>
       </c>
-      <c r="M8" s="32" t="s">
+      <c r="M8" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="N8" s="33">
+      <c r="N8" s="30">
         <v>0.66255669934028294</v>
       </c>
-      <c r="O8" s="32" t="s">
+      <c r="O8" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="P8" s="34" t="s">
+      <c r="P8" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="Q8" s="19">
-        <v>10.02</v>
-      </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>29</v>
       </c>
@@ -1211,50 +1211,47 @@
       <c r="C9" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="27">
+      <c r="E9" s="16">
         <v>0.60099999999999998</v>
       </c>
-      <c r="F9" s="28" t="s">
+      <c r="F9" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="G9" s="27">
+      <c r="G9" s="16">
         <v>0.53500000000000003</v>
       </c>
-      <c r="H9" s="27">
+      <c r="H9" s="16">
         <v>0.247</v>
       </c>
-      <c r="I9" s="27">
+      <c r="I9" s="16">
         <v>0.218</v>
       </c>
-      <c r="J9" s="29">
+      <c r="J9" s="18">
         <v>0.53500000000000003</v>
       </c>
-      <c r="K9" s="30" t="s">
+      <c r="K9" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="L9" s="31">
+      <c r="L9" s="20">
         <v>0.58560000000000001</v>
       </c>
-      <c r="M9" s="32" t="s">
+      <c r="M9" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="N9" s="33">
+      <c r="N9" s="22">
         <v>0.6804794581359136</v>
       </c>
-      <c r="O9" s="26" t="s">
+      <c r="O9" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="P9" s="35" t="s">
+      <c r="P9" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="Q9" s="19">
-        <v>7.66</v>
-      </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>33</v>
       </c>
@@ -1264,50 +1261,47 @@
       <c r="C10" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="26" t="s">
+      <c r="D10" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="E10" s="27">
+      <c r="E10" s="26">
         <v>0.64700000000000002</v>
       </c>
-      <c r="F10" s="28" t="s">
+      <c r="F10" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="27">
+      <c r="G10" s="16">
         <v>0.45700000000000002</v>
       </c>
-      <c r="H10" s="27">
+      <c r="H10" s="16">
         <v>0.30299999999999999</v>
       </c>
-      <c r="I10" s="27">
+      <c r="I10" s="16">
         <v>0.45700000000000002</v>
       </c>
-      <c r="J10" s="29">
+      <c r="J10" s="34">
         <v>0.24099999999999999</v>
       </c>
-      <c r="K10" s="30" t="s">
+      <c r="K10" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="L10" s="31">
+      <c r="L10" s="20">
         <v>0.50280000000000002</v>
       </c>
-      <c r="M10" s="32" t="s">
+      <c r="M10" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="N10" s="33">
+      <c r="N10" s="22">
         <v>0.57766771962853802</v>
       </c>
-      <c r="O10" s="26" t="s">
+      <c r="O10" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="P10" s="35" t="s">
+      <c r="P10" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="Q10" s="19">
-        <v>8.06</v>
-      </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>35</v>
       </c>
@@ -1317,50 +1311,47 @@
       <c r="C11" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="26" t="s">
+      <c r="D11" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="27">
+      <c r="E11" s="26">
         <v>0.57399999999999995</v>
       </c>
-      <c r="F11" s="28" t="s">
+      <c r="F11" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="G11" s="27">
+      <c r="G11" s="26">
         <v>0.54100000000000004</v>
       </c>
-      <c r="H11" s="27">
+      <c r="H11" s="26">
         <v>0.54100000000000004</v>
       </c>
-      <c r="I11" s="27">
+      <c r="I11" s="26">
         <v>0.26300000000000001</v>
       </c>
-      <c r="J11" s="29">
+      <c r="J11" s="28">
         <v>0.19600000000000001</v>
       </c>
-      <c r="K11" s="30" t="s">
+      <c r="K11" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="L11" s="31">
+      <c r="L11" s="20">
         <v>0.50849999999999995</v>
       </c>
-      <c r="M11" s="32" t="s">
+      <c r="M11" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="N11" s="33">
+      <c r="N11" s="30">
         <v>0.52702249019800285</v>
       </c>
-      <c r="O11" s="26" t="s">
+      <c r="O11" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="P11" s="35" t="s">
+      <c r="P11" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="Q11" s="19">
-        <v>11.74</v>
-      </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>37</v>
       </c>
@@ -1370,50 +1361,47 @@
       <c r="C12" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="26" t="s">
+      <c r="D12" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="27">
+      <c r="E12" s="16">
         <v>0.78100000000000003</v>
       </c>
-      <c r="F12" s="28" t="s">
+      <c r="F12" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="G12" s="27">
+      <c r="G12" s="16">
         <v>0.627</v>
       </c>
-      <c r="H12" s="27">
+      <c r="H12" s="16">
         <v>0.2</v>
       </c>
-      <c r="I12" s="27">
+      <c r="I12" s="16">
         <v>0.17299999999999999</v>
       </c>
-      <c r="J12" s="29">
+      <c r="J12" s="18">
         <v>0.627</v>
       </c>
-      <c r="K12" s="30" t="s">
+      <c r="K12" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="L12" s="31">
+      <c r="L12" s="20">
         <v>0.50829999999999997</v>
       </c>
-      <c r="M12" s="32" t="s">
+      <c r="M12" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="N12" s="33">
+      <c r="N12" s="22">
         <v>0.69466768710566251</v>
       </c>
-      <c r="O12" s="26" t="s">
+      <c r="O12" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="P12" s="35" t="s">
+      <c r="P12" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="Q12" s="19">
-        <v>7.52</v>
-      </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>40</v>
       </c>
@@ -1423,50 +1411,47 @@
       <c r="C13" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="26" t="s">
+      <c r="D13" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="E13" s="27">
+      <c r="E13" s="16">
         <v>0.72</v>
       </c>
-      <c r="F13" s="28" t="s">
+      <c r="F13" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="G13" s="27">
+      <c r="G13" s="16">
         <v>0.434</v>
       </c>
-      <c r="H13" s="27">
+      <c r="H13" s="16">
         <v>0.434</v>
       </c>
-      <c r="I13" s="27">
+      <c r="I13" s="16">
         <v>0.34899999999999998</v>
       </c>
-      <c r="J13" s="29">
+      <c r="J13" s="18">
         <v>0.216</v>
       </c>
-      <c r="K13" s="30" t="s">
+      <c r="K13" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="L13" s="31">
+      <c r="L13" s="20">
         <v>0.5413</v>
       </c>
-      <c r="M13" s="32" t="s">
+      <c r="M13" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="N13" s="33">
+      <c r="N13" s="22">
         <v>0.70033629430904631</v>
       </c>
-      <c r="O13" s="32" t="s">
+      <c r="O13" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="P13" s="34" t="s">
+      <c r="P13" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="Q13" s="19">
-        <v>9.83</v>
-      </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>43</v>
       </c>
@@ -1497,26 +1482,23 @@
       <c r="J14" s="9">
         <v>0.17699999999999999</v>
       </c>
-      <c r="K14" s="16" t="s">
+      <c r="K14" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="L14" s="15">
+      <c r="L14" s="12">
         <v>0.62519999999999998</v>
       </c>
-      <c r="M14" s="12" t="s">
+      <c r="M14" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="N14" s="13">
+      <c r="N14" s="32">
         <v>0.53871886983168216</v>
       </c>
-      <c r="O14" s="12" t="s">
+      <c r="O14" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="P14" s="14" t="s">
+      <c r="P14" s="33" t="s">
         <v>17</v>
-      </c>
-      <c r="Q14" s="19">
-        <v>11.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>